<commit_message>
updated test data for date implementation change
</commit_message>
<xml_diff>
--- a/rules/CORE-000658/negative/01/data/unit-test-coreid-FB3412-negative.xlsx
+++ b/rules/CORE-000658/negative/01/data/unit-test-coreid-FB3412-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -49,6 +49,10 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -131,16 +135,17 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -483,24 +488,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>3-4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B3" s="4" t="str">
-        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -518,10 +515,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
@@ -557,122 +554,122 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>RFICDTC</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>2019-03-20</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>RFXSTDTC</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>2018-02-20T09:40</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>RFICDTC</v>
       </c>
-      <c r="F4" s="2" t="str">
-        <v>2018-02-20T11:50</v>
+      <c r="F4" s="4" t="str">
+        <v>2018-02-20T09:41</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>10</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>RFXSTDTC</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>2018-02-20T09:40</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="4">
         <v>11</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>RFICDTC</v>
       </c>
-      <c r="F6" s="2" t="str">
-        <v>2018-02-20T09:50</v>
+      <c r="F6" s="4" t="str">
+        <v>2018-02-21T09:50</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
+      <c r="A7" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="4">
         <v>11</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>RFXSTDTC</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="4" t="str">
         <v>2018-02-20</v>
       </c>
     </row>
@@ -768,802 +765,802 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="7" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="7" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="7" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="7" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="7" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="7" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="7" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="7" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="7" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="6" t="str">
+      <c r="M2" s="7" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="N2" s="7" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="6" t="str">
+      <c r="O2" s="7" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="6" t="str">
+      <c r="P2" s="7" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="6" t="str">
+      <c r="Q2" s="7" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="6" t="str">
+      <c r="R2" s="7" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="6" t="str">
+      <c r="S2" s="7" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="6" t="str">
+      <c r="T2" s="7" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="6" t="str">
+      <c r="U2" s="7" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="6" t="str">
+      <c r="V2" s="7" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="6" t="str">
+      <c r="W2" s="7" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="6" t="str">
+      <c r="X2" s="7" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="Y2" s="6" t="str">
+      <c r="Y2" s="7" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="Z2" s="6" t="str">
+      <c r="Z2" s="7" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="6" t="str">
+      <c r="A3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="7" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="6" t="str">
+      <c r="P3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="7" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="7" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="7">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="7">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="7">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="7">
         <v>4</v>
       </c>
-      <c r="E4" s="6" t="str">
+      <c r="E4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="J4" s="6" t="str">
+      <c r="J4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="K4" s="6" t="str">
+      <c r="K4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="7">
         <v>1</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="7">
         <v>3</v>
       </c>
-      <c r="N4" s="6" t="str">
+      <c r="N4" s="7" t="str">
         <v>19</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="7">
         <v>8</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="7">
         <v>5</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="7">
         <v>1</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4" s="7">
         <v>41</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4" s="7">
         <v>22</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="7">
         <v>8</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="7">
         <v>28</v>
       </c>
-      <c r="V4" s="6">
+      <c r="V4" s="7">
         <v>8</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="7">
         <v>28</v>
       </c>
-      <c r="X4" s="6">
+      <c r="X4" s="7">
         <v>14</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="7">
         <v>200</v>
       </c>
-      <c r="Z4" s="6">
+      <c r="Z4" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>100001</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-01-24</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="K5" s="4" t="str">
-        <v/>
-      </c>
-      <c r="L5" s="4" t="str">
-        <v/>
-      </c>
-      <c r="M5" s="4">
+      <c r="K5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="M5" s="5">
         <v>360001</v>
       </c>
-      <c r="N5" s="4" t="str">
+      <c r="N5" s="5" t="str">
         <v>1954-08-06</v>
       </c>
-      <c r="O5" s="4" t="str">
+      <c r="O5" s="5" t="str">
         <v>63</v>
       </c>
-      <c r="P5" s="4" t="str">
+      <c r="P5" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="4" t="str">
+      <c r="Q5" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="4" t="str">
+      <c r="R5" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="4" t="str">
+      <c r="S5" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="4" t="str">
+      <c r="T5" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U5" s="4" t="str">
+      <c r="U5" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V5" s="4" t="str">
+      <c r="V5" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W5" s="4" t="str">
+      <c r="W5" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X5" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y5" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z5" s="4" t="str">
+      <c r="X5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="5" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>100002</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>2018-04-17T09:25</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>2019-03-13</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="5" t="str">
         <v>2018-04-17T09:25</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>2019-03-13</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-03-22</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2019-09-29</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="5" t="str">
         <v>2019-09-29</v>
       </c>
-      <c r="L6" s="4" t="str">
+      <c r="L6" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>360001</v>
       </c>
-      <c r="N6" s="4" t="str">
+      <c r="N6" s="5" t="str">
         <v>1941-07-03</v>
       </c>
-      <c r="O6" s="4" t="str">
+      <c r="O6" s="5" t="str">
         <v>76</v>
       </c>
-      <c r="P6" s="4" t="str">
+      <c r="P6" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q6" s="4" t="str">
+      <c r="Q6" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R6" s="4" t="str">
+      <c r="R6" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S6" s="4" t="str">
+      <c r="S6" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="4" t="str">
+      <c r="T6" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U6" s="4" t="str">
+      <c r="U6" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V6" s="4" t="str">
+      <c r="V6" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W6" s="4" t="str">
+      <c r="W6" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X6" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y6" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z6" s="4" t="str">
+      <c r="X6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y6" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z6" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="5" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>100003</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>2018-04-18T09:30</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>2018-07-18T11:15</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>2018-04-18T09:30</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>2018-07-18T11:15</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2018-03-22</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="5" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="K7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M7" s="4">
+      <c r="K7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M7" s="5">
         <v>360001</v>
       </c>
-      <c r="N7" s="4" t="str">
+      <c r="N7" s="5" t="str">
         <v>1964-10-28</v>
       </c>
-      <c r="O7" s="4" t="str">
+      <c r="O7" s="5" t="str">
         <v>53</v>
       </c>
-      <c r="P7" s="4" t="str">
+      <c r="P7" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q7" s="4" t="str">
+      <c r="Q7" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R7" s="4" t="str">
+      <c r="R7" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S7" s="4" t="str">
+      <c r="S7" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="4" t="str">
+      <c r="T7" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U7" s="4" t="str">
+      <c r="U7" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V7" s="4" t="str">
+      <c r="V7" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W7" s="4" t="str">
+      <c r="W7" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z7" s="4" t="str">
+      <c r="X7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y7" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z7" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="str">
+      <c r="A8" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="5" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>200004</v>
       </c>
-      <c r="E8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="G8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="H8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I8" s="4" t="str">
+      <c r="E8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="H8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="I8" s="5" t="str">
         <v>2018-04-16</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="5" t="str">
         <v>2018-05-04</v>
       </c>
-      <c r="K8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="L8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="M8" s="4">
+      <c r="K8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M8" s="5">
         <v>360002</v>
       </c>
-      <c r="N8" s="4" t="str">
+      <c r="N8" s="5" t="str">
         <v>1940-08-14</v>
       </c>
-      <c r="O8" s="4" t="str">
+      <c r="O8" s="5" t="str">
         <v>77</v>
       </c>
-      <c r="P8" s="4" t="str">
+      <c r="P8" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q8" s="4" t="str">
+      <c r="Q8" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R8" s="4" t="str">
+      <c r="R8" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S8" s="4" t="str">
+      <c r="S8" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="U8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="V8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="W8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="X8" s="4" t="str">
+      <c r="T8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="U8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="V8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="W8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="X8" s="5" t="str">
         <v>Screen Failure</v>
       </c>
-      <c r="Y8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z8" s="4" t="str">
+      <c r="Y8" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z8" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="str">
+      <c r="A9" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="4" t="str">
+      <c r="B9" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C9" s="4" t="str">
+      <c r="C9" s="5" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>500005</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G9" s="7" t="str">
+      <c r="G9" s="8" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="H9" s="4" t="str">
+      <c r="H9" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I9" s="7" t="str">
+      <c r="I9" s="8" t="str">
         <v>2019-03-20</v>
       </c>
-      <c r="J9" s="4" t="str">
+      <c r="J9" s="5" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="K9" s="4" t="str">
-        <v/>
-      </c>
-      <c r="L9" s="4" t="str">
-        <v/>
-      </c>
-      <c r="M9" s="4">
+      <c r="K9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="M9" s="5">
         <v>500005</v>
       </c>
-      <c r="N9" s="4" t="str">
+      <c r="N9" s="5" t="str">
         <v>1954-08-06</v>
       </c>
-      <c r="O9" s="4" t="str">
+      <c r="O9" s="5" t="str">
         <v>63</v>
       </c>
-      <c r="P9" s="4" t="str">
+      <c r="P9" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q9" s="4" t="str">
+      <c r="Q9" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R9" s="4" t="str">
+      <c r="R9" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S9" s="4" t="str">
+      <c r="S9" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T9" s="4" t="str">
+      <c r="T9" s="5" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="U9" s="4" t="str">
+      <c r="U9" s="5" t="str">
         <v>Placebo</v>
       </c>
-      <c r="V9" s="4" t="str">
+      <c r="V9" s="5" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="W9" s="4" t="str">
+      <c r="W9" s="5" t="str">
         <v>Placebo</v>
       </c>
-      <c r="X9" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y9" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z9" s="4" t="str">
+      <c r="X9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y9" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z9" s="5" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="str">
+      <c r="A10" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B10" s="4" t="str">
+      <c r="B10" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C10" s="4" t="str">
+      <c r="C10" s="5" t="str">
         <v>CDISC006</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <v>600006</v>
       </c>
-      <c r="E10" s="4" t="str">
+      <c r="E10" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="F10" s="4" t="str">
+      <c r="F10" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G10" s="7" t="str">
+      <c r="G10" s="8" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="H10" s="4" t="str">
+      <c r="H10" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I10" s="8" t="str">
-        <v>2018-02-20T11:50</v>
-      </c>
-      <c r="J10" s="4" t="str">
+      <c r="I10" s="9" t="str">
+        <v>2018-02-20T09:41</v>
+      </c>
+      <c r="J10" s="5" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="K10" s="4" t="str">
-        <v/>
-      </c>
-      <c r="L10" s="4" t="str">
-        <v/>
-      </c>
-      <c r="M10" s="4">
+      <c r="K10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="L10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="M10" s="5">
         <v>500005</v>
       </c>
-      <c r="N10" s="4" t="str">
+      <c r="N10" s="5" t="str">
         <v>1954-08-06</v>
       </c>
-      <c r="O10" s="4" t="str">
+      <c r="O10" s="5" t="str">
         <v>63</v>
       </c>
-      <c r="P10" s="4" t="str">
+      <c r="P10" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q10" s="4" t="str">
+      <c r="Q10" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R10" s="4" t="str">
+      <c r="R10" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S10" s="4" t="str">
+      <c r="S10" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T10" s="4" t="str">
+      <c r="T10" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U10" s="4" t="str">
+      <c r="U10" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V10" s="4" t="str">
+      <c r="V10" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W10" s="4" t="str">
+      <c r="W10" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X10" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y10" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z10" s="4" t="str">
+      <c r="X10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y10" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z10" s="5" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="str">
+      <c r="A11" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="4" t="str">
+      <c r="B11" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C11" s="4" t="str">
+      <c r="C11" s="5" t="str">
         <v>CDISC007</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="5">
         <v>700007</v>
       </c>
-      <c r="E11" s="4" t="str">
+      <c r="E11" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="F11" s="4" t="str">
+      <c r="F11" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G11" s="8" t="str">
+      <c r="G11" s="9" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="H11" s="4" t="str">
+      <c r="H11" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I11" s="8" t="str">
-        <v>2018-02-20T09:50</v>
-      </c>
-      <c r="J11" s="4" t="str">
+      <c r="I11" s="9" t="str">
+        <v>2018-02-21T09:50</v>
+      </c>
+      <c r="J11" s="5" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="K11" s="4" t="str">
-        <v/>
-      </c>
-      <c r="L11" s="4" t="str">
-        <v/>
-      </c>
-      <c r="M11" s="4">
+      <c r="K11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="L11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="M11" s="5">
         <v>700007</v>
       </c>
-      <c r="N11" s="4" t="str">
+      <c r="N11" s="5" t="str">
         <v>1954-08-06</v>
       </c>
-      <c r="O11" s="4" t="str">
+      <c r="O11" s="5" t="str">
         <v>63</v>
       </c>
-      <c r="P11" s="4" t="str">
+      <c r="P11" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q11" s="4" t="str">
+      <c r="Q11" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R11" s="4" t="str">
+      <c r="R11" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S11" s="4" t="str">
+      <c r="S11" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T11" s="4" t="str">
+      <c r="T11" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U11" s="4" t="str">
+      <c r="U11" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V11" s="4" t="str">
+      <c r="V11" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W11" s="4" t="str">
+      <c r="W11" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X11" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Y11" s="4" t="str">
-        <v/>
-      </c>
-      <c r="Z11" s="4" t="str">
+      <c r="X11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Y11" s="5" t="str">
+        <v/>
+      </c>
+      <c r="Z11" s="5" t="str">
         <v>USA</v>
       </c>
     </row>

</xml_diff>

<commit_message>
els's comments + deletion of negative/02 test case for absent vars
</commit_message>
<xml_diff>
--- a/rules/CORE-000658/negative/01/data/unit-test-coreid-FB3412-negative.xlsx
+++ b/rules/CORE-000658/negative/01/data/unit-test-coreid-FB3412-negative.xlsx
@@ -534,7 +534,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -634,6 +634,46 @@
       </c>
       <c r="F5" s="2" t="str">
         <v>2018-02-20T09:40</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="2">
+        <v>11</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>RFICDTC</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <v>2018-02-20T09:50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="2">
+        <v>11</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>RFXSTDTC</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>2018-02-20</v>
       </c>
     </row>
   </sheetData>
@@ -1466,13 +1506,13 @@
       <c r="F11" s="4" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G11" t="str" s="4">
+      <c r="G11" s="8" t="str">
         <v>2018-02-20</v>
       </c>
       <c r="H11" s="4" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I11" t="str" s="4">
+      <c r="I11" s="8" t="str">
         <v>2018-02-20T09:50</v>
       </c>
       <c r="J11" s="4" t="str">

</xml_diff>